<commit_message>
docs(pm): walkthrough + charger-view merge decision + matrix refresh
</commit_message>
<xml_diff>
--- a/01需求矩阵-第1组-王浩恩.xlsx
+++ b/01需求矩阵-第1组-王浩恩.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BIT-SummerTermProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AC74975-60AE-452F-9E2D-22F8BA984C0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{859DB534-74A7-433E-BB2E-0CD854393CD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -119,7 +119,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="144">
   <si>
     <t>需求进度管理表</t>
   </si>
@@ -473,13 +473,7 @@
     <t>未开始，今天完成，下周一验收</t>
   </si>
   <si>
-    <t>在 resources/map/navigation.html（已存在于 feat/user）通过 QWebEngineView 加载腾讯地图 JavaScript API GL；接收起点（当前坐标）与终点（电站坐标）显示标记与路线；驾车/步行切换重新规划；失败显示原因与重试，保留最后成功路线缓存。</t>
-  </si>
-  <si>
     <t>11 位手机号正则 ^1[3-9]\d{9}$ 校验；auth.user_login {mobile}；服务端命中即返回 token 直接登录，未命中自动注册为 用户+后4位 并发 token，提示「注册并登录」。</t>
-  </si>
-  <si>
-    <t>登录后展示默认灰色头像、昵称、钱包余额（元）；user.update 改昵称实时落库；wallet.recharge 输入框仅允许两位小数转整数分；头像上传持久化按范围决策不实现（说明书原话答辩时注明）。</t>
   </si>
   <si>
     <t>进入充电页前先调 order.current；若返回 reserved 或 charging 订单弹窗「您有未完成的充电订单，请先结算」并强制跳转当前订单页；否则进入选桩界面。</t>
@@ -585,6 +579,18 @@
       </rPr>
       <t>：已完成</t>
     </r>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>在 resources/map/navigation.html（已存在于 feat/user）通过 QWebEngineView 加载腾讯地图 JavaScript API GL；接收起点（当前坐标）与终点（电站坐标）显示标记与路线；驾车/步行切换重新规划；失败显示原因与重试，保留最后成功路线缓存。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>登录后展示默认灰色头像、昵称、钱包余额（元）；user.update 改昵称实时落库；wallet.recharge 输入框仅允许两位小数转整数分；头像上传持久化按范围决策不实现（说明书原话答辩时注明）。</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>详细说明</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
@@ -999,7 +1005,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="13"/>
     <xf numFmtId="0" fontId="17" fillId="3" borderId="13"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1077,12 +1083,12 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="17" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="3" xfId="17" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="58" fontId="19" fillId="3" borderId="3" xfId="17" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="13" xfId="17" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="17" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1104,8 +1110,20 @@
     <xf numFmtId="58" fontId="3" fillId="3" borderId="5" xfId="17" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="13" xfId="17" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="2" xfId="16" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="3" xfId="17" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="58" fontId="19" fillId="3" borderId="3" xfId="17" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="58" fontId="3" fillId="3" borderId="3" xfId="17" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="13" xfId="17" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="23">
@@ -1602,7 +1620,7 @@
     <col min="3" max="3" width="19.36328125" style="24" customWidth="1"/>
     <col min="4" max="4" width="16.6328125" style="24" customWidth="1"/>
     <col min="5" max="5" width="21.6328125" style="24" customWidth="1"/>
-    <col min="6" max="6" width="57.1796875" style="24" customWidth="1"/>
+    <col min="6" max="6" width="57.1796875" style="40" customWidth="1"/>
     <col min="7" max="7" width="9" style="23" customWidth="1"/>
     <col min="8" max="8" width="10.453125" style="25" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6.36328125" style="25" bestFit="1" customWidth="1"/>
@@ -1611,8 +1629,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="41.25" customHeight="1">
-      <c r="A1" s="36" t="s">
-        <v>142</v>
+      <c r="A1" s="28" t="s">
+        <v>140</v>
       </c>
       <c r="B1" s="29"/>
       <c r="C1" s="29"/>
@@ -1649,8 +1667,8 @@
       <c r="E3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="5" t="s">
-        <v>6</v>
+      <c r="F3" s="36" t="s">
+        <v>143</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>7</v>
@@ -1665,7 +1683,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="4" spans="1:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B4" s="7">
         <v>1</v>
       </c>
@@ -1678,8 +1696,8 @@
       <c r="E4" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="27" t="s">
-        <v>137</v>
+      <c r="F4" s="37" t="s">
+        <v>135</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>14</v>
@@ -1687,12 +1705,12 @@
       <c r="H4" s="10">
         <v>46269</v>
       </c>
-      <c r="I4" s="28" t="s">
-        <v>141</v>
+      <c r="I4" s="27" t="s">
+        <v>139</v>
       </c>
       <c r="J4" s="9"/>
     </row>
-    <row r="5" spans="1:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="5" spans="1:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B5" s="7">
         <v>2</v>
       </c>
@@ -1701,8 +1719,8 @@
       <c r="E5" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="28" t="s">
-        <v>138</v>
+      <c r="F5" s="38" t="s">
+        <v>136</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>14</v>
@@ -1715,7 +1733,7 @@
       </c>
       <c r="J5" s="8"/>
     </row>
-    <row r="6" spans="1:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="6" spans="1:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B6" s="7">
         <v>3</v>
       </c>
@@ -1724,8 +1742,8 @@
       <c r="E6" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="28" t="s">
-        <v>139</v>
+      <c r="F6" s="38" t="s">
+        <v>137</v>
       </c>
       <c r="G6" s="8" t="s">
         <v>14</v>
@@ -1738,7 +1756,7 @@
       </c>
       <c r="J6" s="8"/>
     </row>
-    <row r="7" spans="1:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="7" spans="1:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B7" s="7">
         <v>4</v>
       </c>
@@ -1749,8 +1767,8 @@
       <c r="E7" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="10" t="s">
-        <v>117</v>
+      <c r="F7" s="38" t="s">
+        <v>141</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>14</v>
@@ -1758,12 +1776,12 @@
       <c r="H7" s="10">
         <v>46270</v>
       </c>
-      <c r="I7" s="28" t="s">
-        <v>140</v>
+      <c r="I7" s="27" t="s">
+        <v>138</v>
       </c>
       <c r="J7" s="8"/>
     </row>
-    <row r="8" spans="1:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="8" spans="1:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B8" s="7">
         <v>5</v>
       </c>
@@ -1774,8 +1792,8 @@
       <c r="E8" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="10" t="s">
-        <v>118</v>
+      <c r="F8" s="39" t="s">
+        <v>117</v>
       </c>
       <c r="G8" s="8" t="s">
         <v>14</v>
@@ -1788,7 +1806,7 @@
       </c>
       <c r="J8" s="8"/>
     </row>
-    <row r="9" spans="1:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="9" spans="1:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B9" s="7">
         <v>6</v>
       </c>
@@ -1797,8 +1815,8 @@
       <c r="E9" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="F9" s="10" t="s">
-        <v>119</v>
+      <c r="F9" s="38" t="s">
+        <v>142</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>14</v>
@@ -1811,7 +1829,7 @@
       </c>
       <c r="J9" s="8"/>
     </row>
-    <row r="10" spans="1:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="10" spans="1:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B10" s="7">
         <v>7</v>
       </c>
@@ -1822,8 +1840,8 @@
       <c r="E10" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="F10" s="10" t="s">
-        <v>120</v>
+      <c r="F10" s="39" t="s">
+        <v>118</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>14</v>
@@ -1836,7 +1854,7 @@
       </c>
       <c r="J10" s="8"/>
     </row>
-    <row r="11" spans="1:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="11" spans="1:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B11" s="7">
         <v>8</v>
       </c>
@@ -1845,8 +1863,8 @@
       <c r="E11" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="10" t="s">
-        <v>121</v>
+      <c r="F11" s="39" t="s">
+        <v>119</v>
       </c>
       <c r="G11" s="8" t="s">
         <v>14</v>
@@ -1859,7 +1877,7 @@
       </c>
       <c r="J11" s="8"/>
     </row>
-    <row r="12" spans="1:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="12" spans="1:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B12" s="7">
         <v>9</v>
       </c>
@@ -1872,8 +1890,8 @@
       <c r="E12" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="F12" s="10" t="s">
-        <v>122</v>
+      <c r="F12" s="39" t="s">
+        <v>120</v>
       </c>
       <c r="G12" s="8" t="s">
         <v>30</v>
@@ -1886,7 +1904,7 @@
       </c>
       <c r="J12" s="8"/>
     </row>
-    <row r="13" spans="1:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="13" spans="1:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B13" s="7">
         <v>10</v>
       </c>
@@ -1897,8 +1915,8 @@
       <c r="E13" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="F13" s="10" t="s">
-        <v>123</v>
+      <c r="F13" s="39" t="s">
+        <v>121</v>
       </c>
       <c r="G13" s="8" t="s">
         <v>30</v>
@@ -1911,7 +1929,7 @@
       </c>
       <c r="J13" s="8"/>
     </row>
-    <row r="14" spans="1:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="14" spans="1:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B14" s="7">
         <v>11</v>
       </c>
@@ -1920,8 +1938,8 @@
       <c r="E14" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="F14" s="10" t="s">
-        <v>124</v>
+      <c r="F14" s="39" t="s">
+        <v>122</v>
       </c>
       <c r="G14" s="8" t="s">
         <v>30</v>
@@ -1934,7 +1952,7 @@
       </c>
       <c r="J14" s="8"/>
     </row>
-    <row r="15" spans="1:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="15" spans="1:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B15" s="7">
         <v>12</v>
       </c>
@@ -1945,8 +1963,8 @@
       <c r="E15" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="F15" s="10" t="s">
-        <v>125</v>
+      <c r="F15" s="39" t="s">
+        <v>123</v>
       </c>
       <c r="G15" s="8" t="s">
         <v>30</v>
@@ -1959,7 +1977,7 @@
       </c>
       <c r="J15" s="8"/>
     </row>
-    <row r="16" spans="1:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="16" spans="1:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B16" s="7">
         <v>13</v>
       </c>
@@ -1970,8 +1988,8 @@
       <c r="E16" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="F16" s="10" t="s">
-        <v>126</v>
+      <c r="F16" s="39" t="s">
+        <v>124</v>
       </c>
       <c r="G16" s="8" t="s">
         <v>30</v>
@@ -1984,7 +2002,7 @@
       </c>
       <c r="J16" s="8"/>
     </row>
-    <row r="17" spans="2:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="17" spans="2:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B17" s="7">
         <v>14</v>
       </c>
@@ -1993,8 +2011,8 @@
       <c r="E17" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="F17" s="10" t="s">
-        <v>127</v>
+      <c r="F17" s="39" t="s">
+        <v>125</v>
       </c>
       <c r="G17" s="8" t="s">
         <v>30</v>
@@ -2007,7 +2025,7 @@
       </c>
       <c r="J17" s="8"/>
     </row>
-    <row r="18" spans="2:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="18" spans="2:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B18" s="7">
         <v>15</v>
       </c>
@@ -2018,8 +2036,8 @@
       <c r="E18" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="F18" s="10" t="s">
-        <v>128</v>
+      <c r="F18" s="39" t="s">
+        <v>126</v>
       </c>
       <c r="G18" s="8" t="s">
         <v>30</v>
@@ -2032,7 +2050,7 @@
       </c>
       <c r="J18" s="8"/>
     </row>
-    <row r="19" spans="2:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="19" spans="2:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B19" s="7">
         <v>16</v>
       </c>
@@ -2041,8 +2059,8 @@
       <c r="E19" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="F19" s="10" t="s">
-        <v>129</v>
+      <c r="F19" s="39" t="s">
+        <v>127</v>
       </c>
       <c r="G19" s="8" t="s">
         <v>30</v>
@@ -2055,7 +2073,7 @@
       </c>
       <c r="J19" s="8"/>
     </row>
-    <row r="20" spans="2:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="20" spans="2:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B20" s="7">
         <v>17</v>
       </c>
@@ -2066,8 +2084,8 @@
       <c r="E20" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="F20" s="10" t="s">
-        <v>130</v>
+      <c r="F20" s="39" t="s">
+        <v>128</v>
       </c>
       <c r="G20" s="8" t="s">
         <v>30</v>
@@ -2080,7 +2098,7 @@
       </c>
       <c r="J20" s="8"/>
     </row>
-    <row r="21" spans="2:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="21" spans="2:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B21" s="7">
         <v>18</v>
       </c>
@@ -2089,8 +2107,8 @@
       <c r="E21" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="F21" s="10" t="s">
-        <v>131</v>
+      <c r="F21" s="39" t="s">
+        <v>129</v>
       </c>
       <c r="G21" s="8" t="s">
         <v>30</v>
@@ -2103,7 +2121,7 @@
       </c>
       <c r="J21" s="8"/>
     </row>
-    <row r="22" spans="2:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="22" spans="2:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B22" s="7">
         <v>19</v>
       </c>
@@ -2116,8 +2134,8 @@
       <c r="E22" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="F22" s="10" t="s">
-        <v>132</v>
+      <c r="F22" s="39" t="s">
+        <v>130</v>
       </c>
       <c r="G22" s="8" t="s">
         <v>48</v>
@@ -2130,7 +2148,7 @@
       </c>
       <c r="J22" s="8"/>
     </row>
-    <row r="23" spans="2:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="23" spans="2:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B23" s="7">
         <v>20</v>
       </c>
@@ -2141,8 +2159,8 @@
       <c r="E23" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="F23" s="10" t="s">
-        <v>133</v>
+      <c r="F23" s="39" t="s">
+        <v>131</v>
       </c>
       <c r="G23" s="8" t="s">
         <v>48</v>
@@ -2155,7 +2173,7 @@
       </c>
       <c r="J23" s="8"/>
     </row>
-    <row r="24" spans="2:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="24" spans="2:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B24" s="7">
         <v>21</v>
       </c>
@@ -2168,8 +2186,8 @@
       <c r="E24" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="F24" s="10" t="s">
-        <v>134</v>
+      <c r="F24" s="39" t="s">
+        <v>132</v>
       </c>
       <c r="G24" s="8" t="s">
         <v>54</v>
@@ -2182,7 +2200,7 @@
       </c>
       <c r="J24" s="8"/>
     </row>
-    <row r="25" spans="2:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="25" spans="2:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B25" s="7">
         <v>22</v>
       </c>
@@ -2195,8 +2213,8 @@
       <c r="E25" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="F25" s="10" t="s">
-        <v>135</v>
+      <c r="F25" s="39" t="s">
+        <v>133</v>
       </c>
       <c r="G25" s="8" t="s">
         <v>58</v>
@@ -2209,7 +2227,7 @@
       </c>
       <c r="J25" s="8"/>
     </row>
-    <row r="26" spans="2:10" s="23" customFormat="1" ht="31.5" customHeight="1">
+    <row r="26" spans="2:10" s="23" customFormat="1" ht="128.5" customHeight="1">
       <c r="B26" s="7">
         <v>23</v>
       </c>
@@ -2218,8 +2236,8 @@
       <c r="E26" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="F26" s="10" t="s">
-        <v>136</v>
+      <c r="F26" s="39" t="s">
+        <v>134</v>
       </c>
       <c r="G26" s="8" t="s">
         <v>58</v>

</xml_diff>